<commit_message>
Whitepaper and BOE carry the layer escalators and the savings register; BLS escalator series pulled from the FRED and BLS APIs
- Whitepaper: new 5.3 (one escalator per layer, methods table, scaling recipe), new 8 (savings register, tier totals, Section 48E), recommendations extended, sources appended
- BOE: escalator check in 1.3 and 14 (template 3%/yr vs the published series 2023-2026), risk-register overlap in 18, E&S basis question in 19, AFUDC timing in 20, six new open items in 22
- fetch_indices.py now uses the keyless FRED CSV and BLS v2 endpoints; indices_layers_api.json holds ten BLS series 2014-2026 and overrides the search-excerpt values (results unchanged: composite 1.17x, class median $832)
- Breaker lever sized on the furnish line only; README and research log updated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YAU7MDk5K6GEm6c4td5TUq
</commit_message>
<xml_diff>
--- a/Hyde Park BESS/6) Cost Analysis Deliverables/Hyde Park BESS - Cost Analysis Workbook.xlsx
+++ b/Hyde Park BESS/6) Cost Analysis Deliverables/Hyde Park BESS - Cost Analysis Workbook.xlsx
@@ -4264,7 +4264,7 @@
     <t xml:space="preserve">Budgetary quote for the SDV7-class breaker with relay cabinet; confirm what the project team's number includes</t>
   </si>
   <si>
-    <t xml:space="preserve">Four at $374K furnish. A Siemens SDV7-SE 1200 A lists at about $50K (distributor listings, Medium-Low); Siemens has quoted the skids, so the question is what the skid price includes.</t>
+    <t xml:space="preserve">Four at $332K furnish. A Siemens SDV7-SE 1200 A lists at about $50K (distributor listings, Medium-Low); Siemens has quoted the skids, so the question is what the skid price includes.</t>
   </si>
   <si>
     <t xml:space="preserve">B6</t>
@@ -10270,7 +10270,7 @@
         <v>832</v>
       </c>
       <c r="C40" s="58" t="n">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D40" s="58" t="n">
         <v>1163</v>
@@ -10282,7 +10282,7 @@
         <v>0.854545454545455</v>
       </c>
       <c r="G40" s="58" t="n">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="H40" s="62" t="n">
         <v>0.741935483870968</v>
@@ -10296,22 +10296,22 @@
         <v>832</v>
       </c>
       <c r="C41" s="58" t="n">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D41" s="58" t="n">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="E41" s="62" t="n">
         <v>0.509090909090909</v>
       </c>
       <c r="F41" s="62" t="n">
-        <v>0.836363636363636</v>
+        <v>0.854545454545455</v>
       </c>
       <c r="G41" s="58" t="n">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="H41" s="62" t="n">
-        <v>0.709677419354839</v>
+        <v>0.741935483870968</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10319,22 +10319,22 @@
         <v>1248</v>
       </c>
       <c r="B42" s="58" t="n">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C42" s="58" t="n">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D42" s="58" t="n">
         <v>1190</v>
       </c>
       <c r="E42" s="62" t="n">
-        <v>0.563636363636364</v>
+        <v>0.545454545454545</v>
       </c>
       <c r="F42" s="62" t="n">
         <v>0.872727272727273</v>
       </c>
       <c r="G42" s="58" t="n">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="H42" s="62" t="n">
         <v>0.774193548387097</v>
@@ -10345,10 +10345,10 @@
         <v>1249</v>
       </c>
       <c r="B43" s="58" t="n">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C43" s="58" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D43" s="58" t="n">
         <v>1108</v>
@@ -10360,7 +10360,7 @@
         <v>0.890909090909091</v>
       </c>
       <c r="G43" s="58" t="n">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="H43" s="62" t="n">
         <v>0.806451612903226</v>
@@ -11461,21 +11461,21 @@
         <v>1394</v>
       </c>
       <c r="E17" s="69" t="n">
-        <v>299326</v>
+        <v>265476</v>
       </c>
       <c r="F17" s="69" t="n">
-        <v>598652</v>
+        <v>530952</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>1</v>
       </c>
       <c r="H17" s="71" t="n">
         <f aca="false">E17*IF(G17=1,$B$4,1)</f>
-        <v>431029.44</v>
+        <v>382285.44</v>
       </c>
       <c r="I17" s="71" t="n">
         <f aca="false">F17*IF(G17=1,$B$4,1)</f>
-        <v>862058.88</v>
+        <v>764570.88</v>
       </c>
       <c r="J17" s="68" t="s">
         <v>196</v>
@@ -11689,19 +11689,19 @@
       </c>
       <c r="E24" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"B",E8:E21)</f>
-        <v>3317553</v>
+        <v>3283703</v>
       </c>
       <c r="F24" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"B",F8:F21)</f>
-        <v>5309592</v>
+        <v>5241892</v>
       </c>
       <c r="H24" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"B",H8:H21)</f>
-        <v>4308283.84</v>
+        <v>4259539.84</v>
       </c>
       <c r="I24" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"B",I8:I21)</f>
-        <v>6975823.16</v>
+        <v>6878335.16</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11731,11 +11731,11 @@
       </c>
       <c r="H26" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"A",H8:H21)+SUMIF($B$8:$B$21,"B",H8:H21)</f>
-        <v>9320712.04</v>
+        <v>9271968.04</v>
       </c>
       <c r="I26" s="72" t="n">
         <f aca="false">SUMIF($B$8:$B$21,"A",I8:I21)+SUMIF($B$8:$B$21,"B",I8:I21)</f>
-        <v>14122162.36</v>
+        <v>14024674.36</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>